<commit_message>
Add backward compatibility filling from default dictionary
</commit_message>
<xml_diff>
--- a/Work/Test_setup.xlsx
+++ b/Work/Test_setup.xlsx
@@ -5,19 +5,19 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Denise/Library/CloudStorage/Dropbox/Postcard Files/ROVPrograms/cleaver-root/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Denise/Library/CloudStorage/Dropbox/Postcard Files/ROVPrograms/cleaver-root/Work/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37B94B7E-D944-5847-98B0-318F025A7DBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDDF664A-A9BA-2747-91DF-A0F7C232BA88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3700" yWindow="3740" windowWidth="27640" windowHeight="16680" activeTab="1" xr2:uid="{6D162710-0004-644E-A22E-C611B019609F}"/>
+    <workbookView xWindow="2280" yWindow="1540" windowWidth="27640" windowHeight="16680" activeTab="1" xr2:uid="{6D162710-0004-644E-A22E-C611B019609F}"/>
   </bookViews>
   <sheets>
     <sheet name="Setup" sheetId="1" r:id="rId1"/>
     <sheet name="FileList" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">FileList!$A$3:$G$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">FileList!$A$3:$G$3</definedName>
     <definedName name="postfix">#REF!</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Setup!$G$1:$L$192</definedName>
     <definedName name="state">#REF!</definedName>
@@ -531,7 +531,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="281">
   <si>
     <t>dummyCol</t>
   </si>
@@ -1343,9 +1343,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>2026 General Accomack.csv</t>
-  </si>
-  <si>
     <t>x</t>
   </si>
   <si>
@@ -1358,76 +1355,52 @@
     <t>5</t>
   </si>
   <si>
-    <t>CD5. Pulled 6/17/26.</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
     <t>1</t>
   </si>
   <si>
-    <t>CD7. NOVA. Pulled 6/17/26.</t>
-  </si>
-  <si>
-    <t>NoVA</t>
-  </si>
-  <si>
-    <t>2026 General Goochland.csv</t>
-  </si>
-  <si>
-    <t>2026 General Hanover CD1.csv</t>
-  </si>
-  <si>
-    <t>REMOVED - DUPE. Pulled 6/9/26. CD1.  Was honover.xlsx; CD1 added to file name in rawdata/xlsx</t>
-  </si>
-  <si>
-    <t>2026 General Hanover CD5.csv</t>
-  </si>
-  <si>
-    <t>REMOVED - DUPE. Pulled 6/9/26. CD5.  Was honover (1).xlsx; CD5 added to file name in rawdata/xlsx</t>
-  </si>
-  <si>
-    <t>2026 General Hanover(1).csv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CD 1&amp;5. Pulled 6/23/26 by county, not CD.  Replaced two dupe files. </t>
-  </si>
-  <si>
-    <t>2026 General Isle of Wight.csv</t>
-  </si>
-  <si>
-    <t>2026 General Northampton (1).csv</t>
-  </si>
-  <si>
-    <t>CD2. Pulled 6/9/26. No Northampton.xlsx wo "(1)"</t>
-  </si>
-  <si>
-    <t>2026 General Prince William.csv</t>
-  </si>
-  <si>
-    <t>2026 General Northampton(1).csv</t>
-  </si>
-  <si>
-    <t>2026 General Hanover.csv</t>
-  </si>
-  <si>
-    <t>2026 Special General Accomack.csv</t>
-  </si>
-  <si>
-    <t>2026     General Accomack.csv</t>
-  </si>
-  <si>
-    <t>2026     General Accomack Remainder.csv</t>
-  </si>
-  <si>
-    <t>2026 General Accccccomack.csv</t>
-  </si>
-  <si>
-    <t>2026 General Roanoke.csv</t>
-  </si>
-  <si>
-    <t>2026 General Roanoke City.csv</t>
+    <t>2026 General Madison.csv</t>
+  </si>
+  <si>
+    <t>2026 General Maaaaadison.csv</t>
+  </si>
+  <si>
+    <t>2026 Special General Madison.csv</t>
+  </si>
+  <si>
+    <t>2026  General  Madison.csv</t>
+  </si>
+  <si>
+    <t>2026- General-Madison.csv</t>
+  </si>
+  <si>
+    <t>2026 General Madison All.csv</t>
+  </si>
+  <si>
+    <t>2026 General Madison (1).csv</t>
+  </si>
+  <si>
+    <t>2026 General Madison(1).csv</t>
+  </si>
+  <si>
+    <t>2026 General Madison 1.csv</t>
+  </si>
+  <si>
+    <t>2026 General King and Queen.xlsx</t>
+  </si>
+  <si>
+    <t>2026 General James City.xlsx</t>
+  </si>
+  <si>
+    <t>2026 General Virginia Beach.xlsx</t>
+  </si>
+  <si>
+    <t>2026 General Richmond City.xlsx</t>
+  </si>
+  <si>
+    <t>2026 General Richmond County.xlsx</t>
+  </si>
+  <si>
+    <t>2026 General Richmond.xlsx</t>
   </si>
 </sst>
 </file>
@@ -1438,7 +1411,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(\ #,##0_);_(\ \(#,##0\);_(&quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1587,14 +1560,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -1706,7 +1671,7 @@
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1799,21 +1764,6 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -4656,7 +4606,7 @@
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
@@ -4664,7 +4614,7 @@
     <col min="3" max="3" width="14.6640625" style="20" customWidth="1"/>
     <col min="4" max="4" width="29.1640625" style="20" bestFit="1" customWidth="1"/>
     <col min="5" max="7" width="14.6640625" style="20" customWidth="1"/>
-    <col min="8" max="8" width="24" style="58" customWidth="1"/>
+    <col min="8" max="8" width="24" style="53" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="17" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -4719,102 +4669,87 @@
     </row>
     <row r="4" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>266</v>
+      </c>
+      <c r="B4" s="20" t="s">
         <v>261</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="C4" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="G4" s="20" t="s">
         <v>262</v>
       </c>
-      <c r="C4" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="F4" s="20">
-        <v>1</v>
-      </c>
-      <c r="G4" s="20" t="s">
+      <c r="H4" t="s">
         <v>263</v>
-      </c>
-      <c r="H4" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>287</v>
+        <v>267</v>
       </c>
       <c r="B5" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="G5" s="20" t="s">
         <v>262</v>
       </c>
-      <c r="C5" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="F5" s="20">
-        <v>1</v>
-      </c>
-      <c r="G5" s="20" t="s">
+      <c r="H5" t="s">
         <v>263</v>
-      </c>
-      <c r="H5" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>284</v>
+        <v>268</v>
       </c>
       <c r="B6" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="G6" s="20" t="s">
         <v>262</v>
       </c>
-      <c r="C6" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="F6" s="20">
-        <v>1</v>
-      </c>
-      <c r="G6" s="20" t="s">
+      <c r="H6" t="s">
         <v>263</v>
-      </c>
-      <c r="H6" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>285</v>
+        <v>269</v>
       </c>
       <c r="B7" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="G7" s="20" t="s">
         <v>262</v>
       </c>
-      <c r="C7" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="F7" s="20">
-        <v>1</v>
-      </c>
-      <c r="G7" s="20" t="s">
+      <c r="H7" t="s">
         <v>263</v>
-      </c>
-      <c r="H7" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>286</v>
+        <v>270</v>
       </c>
       <c r="B8" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="G8" s="20" t="s">
         <v>262</v>
       </c>
-      <c r="C8" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="F8" s="20">
-        <v>1</v>
-      </c>
-      <c r="G8" s="20" t="s">
+      <c r="H8" t="s">
         <v>263</v>
-      </c>
-      <c r="H8" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15" x14ac:dyDescent="0.2">
@@ -4822,268 +4757,176 @@
         <v>271</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="F9" s="20">
-        <v>1</v>
+        <v>261</v>
       </c>
       <c r="G9" s="20" t="s">
+        <v>264</v>
+      </c>
+      <c r="H9" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>272</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="G10" s="20" t="s">
         <v>265</v>
       </c>
-      <c r="H9" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" s="46" t="s">
-        <v>283</v>
-      </c>
-      <c r="B10" s="53"/>
-      <c r="C10" s="53"/>
-      <c r="F10" s="20">
-        <v>1</v>
-      </c>
-      <c r="G10" s="20" t="s">
-        <v>268</v>
-      </c>
-      <c r="H10" s="56" t="s">
+      <c r="H10" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" s="46" t="s">
-        <v>272</v>
-      </c>
-      <c r="B11" s="53"/>
-      <c r="C11" s="53"/>
-      <c r="F11" s="20">
-        <v>1</v>
+      <c r="B11" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>261</v>
       </c>
       <c r="G11" s="20" t="s">
-        <v>268</v>
-      </c>
-      <c r="H11" s="56" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" s="46" t="s">
+        <v>265</v>
+      </c>
+      <c r="H11" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>274</v>
       </c>
-      <c r="B12" s="53"/>
-      <c r="C12" s="53"/>
-      <c r="F12" s="20">
-        <v>1</v>
+      <c r="B12" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>261</v>
       </c>
       <c r="G12" s="20" t="s">
-        <v>265</v>
-      </c>
-      <c r="H12" s="56" t="s">
+        <v>264</v>
+      </c>
+      <c r="H12" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>276</v>
-      </c>
       <c r="B13" s="20" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="F13" s="20">
-        <v>1</v>
+        <v>261</v>
       </c>
       <c r="G13" s="20">
         <v>15</v>
       </c>
-      <c r="H13" s="57" t="s">
-        <v>277</v>
+      <c r="H13" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B14" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="G14" s="20" t="s">
         <v>262</v>
       </c>
-      <c r="C14" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="F14" s="20">
-        <v>1</v>
-      </c>
-      <c r="G14" s="20" t="s">
+      <c r="H14" t="s">
         <v>263</v>
-      </c>
-      <c r="H14" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B15" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="C15" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="G15" s="20" t="s">
         <v>262</v>
       </c>
-      <c r="C15" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="F15" s="20">
-        <v>1</v>
-      </c>
-      <c r="G15" s="20" t="s">
+      <c r="H15" t="s">
         <v>263</v>
-      </c>
-      <c r="H15" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="B16" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="G16" s="20" t="s">
         <v>262</v>
       </c>
-      <c r="C16" s="20" t="s">
+      <c r="H16" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>279</v>
+      </c>
+      <c r="B17" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="C17" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="G17" s="20" t="s">
         <v>262</v>
       </c>
-      <c r="F16" s="20">
-        <v>1</v>
-      </c>
-      <c r="G16" s="20" t="s">
+      <c r="H17" t="s">
         <v>263</v>
       </c>
-      <c r="H16" t="s">
+    </row>
+    <row r="18" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A17" s="47" t="s">
-        <v>281</v>
-      </c>
-      <c r="B17" s="53"/>
-      <c r="C17" s="53"/>
-      <c r="D17" s="54"/>
-      <c r="E17" s="54"/>
-      <c r="F17" s="54">
-        <v>1</v>
-      </c>
-      <c r="G17" s="54" t="s">
-        <v>267</v>
-      </c>
-      <c r="H17" s="47" t="s">
-        <v>269</v>
-      </c>
-      <c r="I17" s="47"/>
-      <c r="J17" s="47"/>
-      <c r="K17" s="55" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>288</v>
-      </c>
       <c r="B18" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="C18" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="G18" s="20" t="s">
         <v>262</v>
       </c>
-      <c r="C18" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="F18" s="20">
-        <v>1</v>
-      </c>
-      <c r="G18" s="20" t="s">
+      <c r="H18" t="s">
         <v>263</v>
       </c>
-      <c r="H18" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>289</v>
-      </c>
-      <c r="B19" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="C19" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="F19" s="20">
-        <v>1</v>
-      </c>
-      <c r="G19" s="20" t="s">
-        <v>263</v>
-      </c>
-      <c r="H19" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="H19"/>
+    </row>
+    <row r="20" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="H20"/>
-    </row>
-    <row r="21" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="H21"/>
-    </row>
-    <row r="22" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="H22"/>
-    </row>
-    <row r="23" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="H23"/>
-    </row>
-    <row r="24" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="H24"/>
-    </row>
-    <row r="25" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="H25"/>
-    </row>
-    <row r="26" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="H26"/>
-    </row>
-    <row r="27" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="H27"/>
-    </row>
-    <row r="28" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="H28"/>
-    </row>
-    <row r="29" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="H29"/>
-    </row>
-    <row r="30" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="H30"/>
-    </row>
-    <row r="31" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="H31"/>
-    </row>
-    <row r="32" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="H32"/>
-    </row>
-    <row r="33" spans="8:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="H33"/>
-    </row>
-    <row r="34" spans="8:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="H34"/>
-    </row>
-    <row r="35" spans="8:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="H35"/>
-    </row>
-    <row r="36" spans="8:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="H36"/>
-    </row>
-    <row r="37" spans="8:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="H37"/>
-    </row>
-    <row r="38" spans="8:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="H38"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>